<commit_message>
Harmonization - Step 5 - Plots
</commit_message>
<xml_diff>
--- a/dictionary/variables_master.xlsx
+++ b/dictionary/variables_master.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eafit-my.sharepoint.com/personal/rszapatav_eafit_edu_co/Documents/CIAT/Metodología Evaluaciones/surveyProcessingMethodology/dictionary/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="891" documentId="8_{4C1B0862-69B3-42BC-8750-06EDE6596D4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C2198CE4-74E4-4C57-A05D-2C02807DFB34}"/>
+  <xr:revisionPtr revIDLastSave="904" documentId="8_{4C1B0862-69B3-42BC-8750-06EDE6596D4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{71673B79-A3F3-41A9-A8FE-5CA76434128A}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-4725" windowWidth="29040" windowHeight="15720" xr2:uid="{D5E2868F-FAC0-444C-BFCE-6871238D4C9E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{D5E2868F-FAC0-444C-BFCE-6871238D4C9E}"/>
   </bookViews>
   <sheets>
     <sheet name="variables_master" sheetId="2" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="218">
   <si>
     <t>variable_name</t>
   </si>
@@ -675,13 +675,19 @@
     <t>plots</t>
   </si>
   <si>
-    <t>grouping_var</t>
-  </si>
-  <si>
-    <t>logarithm</t>
-  </si>
-  <si>
-    <t>model_var</t>
+    <t>outcome_var</t>
+  </si>
+  <si>
+    <t>control_var</t>
+  </si>
+  <si>
+    <t>logarithm_var</t>
+  </si>
+  <si>
+    <t>fe_var</t>
+  </si>
+  <si>
+    <t>cluster_var</t>
   </si>
 </sst>
 </file>
@@ -1644,7 +1650,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B98D0170-56BF-40AD-B5DE-47C0DB191985}">
-  <dimension ref="A1:AB28"/>
+  <dimension ref="A1:AD28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.140625" customWidth="1"/>
@@ -1668,11 +1674,14 @@
     <col min="20" max="20" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="17.28515625" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="19" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="10.42578125" customWidth="1"/>
+    <col min="30" max="30" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>3</v>
       </c>
@@ -1748,17 +1757,23 @@
       <c r="Y1" s="11" t="s">
         <v>212</v>
       </c>
-      <c r="Z1" s="11" t="s">
+      <c r="Z1" s="12" t="s">
         <v>213</v>
       </c>
       <c r="AA1" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="AB1" s="12" t="s">
         <v>215</v>
       </c>
-      <c r="AB1" s="12" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC1" s="12" t="s">
+        <v>216</v>
+      </c>
+      <c r="AD1" s="12" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>159</v>
       </c>
@@ -1810,8 +1825,14 @@
       <c r="AB2">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC2">
+        <v>0</v>
+      </c>
+      <c r="AD2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>159</v>
       </c>
@@ -1863,8 +1884,14 @@
       <c r="AB3">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC3">
+        <v>0</v>
+      </c>
+      <c r="AD3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>159</v>
       </c>
@@ -1922,8 +1949,14 @@
       <c r="AB4">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC4">
+        <v>0</v>
+      </c>
+      <c r="AD4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>159</v>
       </c>
@@ -1978,8 +2011,14 @@
       <c r="AB5">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC5">
+        <v>0</v>
+      </c>
+      <c r="AD5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>159</v>
       </c>
@@ -2037,8 +2076,14 @@
       <c r="AB6">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC6">
+        <v>0</v>
+      </c>
+      <c r="AD6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -2108,8 +2153,14 @@
       <c r="AB7">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC7">
+        <v>0</v>
+      </c>
+      <c r="AD7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -2170,8 +2221,14 @@
       <c r="AB8">
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC8">
+        <v>0</v>
+      </c>
+      <c r="AD8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -2241,8 +2298,14 @@
       <c r="AB9">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC9">
+        <v>0</v>
+      </c>
+      <c r="AD9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -2312,8 +2375,14 @@
       <c r="AB10">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC10">
+        <v>0</v>
+      </c>
+      <c r="AD10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -2371,8 +2440,14 @@
       <c r="AB11">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC11">
+        <v>0</v>
+      </c>
+      <c r="AD11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -2439,8 +2514,14 @@
       <c r="AB12">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC12">
+        <v>0</v>
+      </c>
+      <c r="AD12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>21</v>
       </c>
@@ -2499,8 +2580,14 @@
       <c r="AB13">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC13">
+        <v>0</v>
+      </c>
+      <c r="AD13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>21</v>
       </c>
@@ -2564,8 +2651,14 @@
       <c r="AB14">
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC14">
+        <v>0</v>
+      </c>
+      <c r="AD14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>21</v>
       </c>
@@ -2626,8 +2719,14 @@
       <c r="AB15">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC15">
+        <v>0</v>
+      </c>
+      <c r="AD15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>21</v>
       </c>
@@ -2700,8 +2799,14 @@
       <c r="AB16">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC16">
+        <v>0</v>
+      </c>
+      <c r="AD16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>21</v>
       </c>
@@ -2769,8 +2874,14 @@
       <c r="AB17">
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC17">
+        <v>0</v>
+      </c>
+      <c r="AD17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>21</v>
       </c>
@@ -2838,8 +2949,14 @@
       <c r="AB18">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC18">
+        <v>0</v>
+      </c>
+      <c r="AD18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>21</v>
       </c>
@@ -2909,8 +3026,14 @@
       <c r="AB19">
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC19">
+        <v>0</v>
+      </c>
+      <c r="AD19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>21</v>
       </c>
@@ -2981,8 +3104,14 @@
       <c r="AB20">
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC20">
+        <v>0</v>
+      </c>
+      <c r="AD20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>21</v>
       </c>
@@ -3040,8 +3169,14 @@
       <c r="AB21">
         <v>0</v>
       </c>
-    </row>
-    <row r="22" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC21">
+        <v>0</v>
+      </c>
+      <c r="AD21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>173</v>
       </c>
@@ -3102,8 +3237,14 @@
       <c r="AB22">
         <v>0</v>
       </c>
-    </row>
-    <row r="23" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC22">
+        <v>0</v>
+      </c>
+      <c r="AD22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>173</v>
       </c>
@@ -3158,8 +3299,14 @@
       <c r="AB23">
         <v>0</v>
       </c>
-    </row>
-    <row r="24" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC23">
+        <v>0</v>
+      </c>
+      <c r="AD23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>173</v>
       </c>
@@ -3217,8 +3364,14 @@
       <c r="AB24">
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC24">
+        <v>0</v>
+      </c>
+      <c r="AD24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>173</v>
       </c>
@@ -3288,8 +3441,14 @@
       <c r="AB25">
         <v>0</v>
       </c>
-    </row>
-    <row r="26" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC25">
+        <v>0</v>
+      </c>
+      <c r="AD25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>173</v>
       </c>
@@ -3356,8 +3515,14 @@
       <c r="AB26">
         <v>0</v>
       </c>
-    </row>
-    <row r="27" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC26">
+        <v>0</v>
+      </c>
+      <c r="AD26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>173</v>
       </c>
@@ -3418,8 +3583,14 @@
       <c r="AB27">
         <v>0</v>
       </c>
-    </row>
-    <row r="28" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC27">
+        <v>0</v>
+      </c>
+      <c r="AD27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>155</v>
       </c>
@@ -3478,6 +3649,12 @@
         <v>0</v>
       </c>
       <c r="AB28">
+        <v>0</v>
+      </c>
+      <c r="AC28">
+        <v>0</v>
+      </c>
+      <c r="AD28">
         <v>0</v>
       </c>
     </row>

</xml_diff>